<commit_message>
pipi popopop json type shti fr rr  frfr
</commit_message>
<xml_diff>
--- a/shap_values_explained.xlsx
+++ b/shap_values_explained.xlsx
@@ -1050,7 +1050,7 @@
       </c>
       <c r="BQ2" t="inlineStr">
         <is>
-          <t>The score for this customer (cust_1000) was heavily influenced by the negative impact of their Usage Frequency, which contributed a significant -1.4805 points to the overall score. This suggests that the customer's usage habits may not be aligned with our desired behavior. Additionally, other factors such as Page Views and Product Views also had a negative impact, contributing another -3.8454 points. Overall, the net impact of these contributions was a score of 0.0100, indicating a relatively low score.</t>
+          <t>The model score for this customer (cust_1000) is 0.0100, with a net impact of -6.8680. The dominant factor contributing to the negative score is Usage Frequency (-1.4805), which accounts for approximately 6% of the total negative impact. This suggests that the customer's usage frequency had a significant negative influence on their overall score.</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="BQ3" t="inlineStr">
         <is>
-          <t>The top contributor to this score is API Calls, which had a positive impact of +1.4686. This suggests that the customer's interactions with our application were a significant factor in determining their overall score. In fact, the dominant feature was API Calls, making up 6.7% of the total contribution. The net impact of all contributors was -1.8005, indicating a slightly negative tilt. However, the positive contributions from API Calls and other factors like Page Views (+1.4193) and Churn Risk (+1.3100) helped to balance out the overall score.</t>
+          <t>The dominant factor driving the model score of 0.3411 is API Calls, which had a positive contribution of +1.4686. This suggests that the customer's behavior in terms of API usage was a significant influencer of their overall score. While there were an equal number of positive and negative contributors, the net impact was slightly negative at -1.8005 due to larger negative contributions from Ad Impressions (-1.3625) and Product Views (-1.2606).</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="BQ4" t="inlineStr">
         <is>
-          <t>The model score for this customer (cust_1002) is 0.2910, indicating a moderate influence on the overall score. The top contributor to this score is Engagement Rate, with a positive value of +1.4926, which suggests that the customer's engagement level had a significant impact on their score. This is likely due to the fact that the customer spent more time interacting with our content and features, which positively influenced their overall score.</t>
+          <t>The model score for this customer (cust_1002) is 0.2910, with a net impact of -2.2029. The dominant factor driving the negative score is Engagement Rate (-1.4926), which accounts for 6.5% of the total contribution. This suggests that while the customer engaged with our content, it wasn't enough to overcome other negative factors such as Time on Site (-1.4037) and Newsletter Signup (-1.3587).</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="BQ5" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1003" who received an email on April 11, 2024, and made a purchase worth $1763.51, the model score is 0.6574. The top contributor to this score is actually negative, which is Trial Conversions (-1.4983). This suggests that the customer's lack of trial conversions had a significant impact on their overall score. However, there were also some positive contributors, such as Page Views (+1.4132) and Product Views (+1.3614), which helped to offset the negative effect. Overall, the net impact is +1.2882, indicating that this customer's behavior was slightly more positive than negative.</t>
+          <t>The dominant factor driving the model score of 0.6574 for customer cust_1003 is the negative impact from Trial Conversions, which contributed -1.4983 to the total score. This suggests that the customer's lack of trial conversions had a significant influence on their overall score. However, it's worth noting that the positive contributions from Page Views (+1.4132) and Product Views (+1.3614) helped mitigate this negative impact, resulting in a net impact of +1.2882. Overall, the customer's behavior was slightly tilted towards a positive outcome, driven by their engagement with product-related features.</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="BQ6" t="inlineStr">
         <is>
-          <t>The top contributor to this score is Usage Frequency, with a positive impact of +1.4854. This suggests that the customer's frequency of using our product or service had a significant influence on their overall score. In fact, it was the dominant factor, making up 6.7% of the total contribution. The other top contributors were also related to usage and engagement, such as Email Opens and Page Views. Overall, the net impact of these contributions is negative (-5.5432), indicating that while some factors had a positive influence, others had a more significant negative effect.</t>
+          <t>The model score for this customer (cust_1004) is 0.0100, which was influenced by a net negative impact of -5.5432. The dominant factor contributing to this score is Usage Frequency (+1.4854), accounting for approximately 6.7% of the total contribution. This suggests that the customer's usage frequency had a significant positive impact on their model score.</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="BQ7" t="inlineStr">
         <is>
-          <t>The top contributor to this score is Usage Frequency, with a positive value of +1.4525. This suggests that the customer's frequent usage of our product or service had a significant impact on their overall score. In fact, the dominant feature in this case is Usage Frequency, which accounts for 6.6% of the total contribution. The net impact of these contributions is a negative value of -2.4118, indicating that while some factors positively influenced the score, others had a more significant negative effect. Overall, it appears that the customer's usage habits played a crucial role in shaping their score.</t>
+          <t>The model score for customer cust_1005, who interacted with our brand through the Direct channel and is part of the SMB segment, was 0.2873. The dominant factor driving this score is Usage Frequency, which had a positive contribution of +1.4525. This suggests that the customer's frequent engagement with our content and features had a significant impact on their overall model score. While there were some negative contributors, such as Email Opens (-1.2874) and Cart Abandonment (-1.2092), the net impact was still slightly negative at -2.4118. Overall, the customer's high usage frequency was the key driver of their model score.</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="BQ8" t="inlineStr">
         <is>
-          <t>The model score for this customer (cust_1006) is 0.9900, indicating a strong positive influence on the purchase decision. The top contributor to this score is Page Views (+1.4978), which had a significant impact on the overall outcome. This suggests that the customer's engagement with our website content was a key factor in their decision to make a purchase. Additionally, Plan Type (+1.4863) and Product Views (+1.4559) also played important roles. Overall, the net impact of these factors is positive, with a total positive contribution of +15.0022 and no negative contributors.</t>
+          <t>The model score for customer cust_1006, who made a purchase on 2024-07-30 through the Social channel and belongs to the SMB segment, is 0.9900. The dominant factor driving this score is Page Views, which contributed +1.4978 points, accounting for 6.2% of the total positive impact. Overall, the net impact is +5.7225, indicating a strong positive influence from various features, with most contributors being positive (17 out of 24).</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="BQ9" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1007" who interacted with our Paid Ad on August 14, 2024, the model score is 0.0408. The top contributors to this score are Engagement Rate (-1.4721) and Form Submissions (-1.3808), which had a net negative impact of -4.7057. This suggests that while there were some positive interactions with our ad (such as Purchase History +1.3248 and Churn Risk +1.3072), the overall influence was driven by lower engagement rates and fewer form submissions, resulting in a negative score.</t>
+          <t>The model score for this customer, cust_1007, is 0.0408, which indicates a relatively low overall impact. The dominant factor driving this result is the Engagement Rate, with a negative contribution of -1.4721, making up about 6.6% of the total impact. This suggests that the lack of engagement from this customer was a significant detractor. Additionally, Form Submissions and Email Opens also had negative contributions, while Purchase History and Churn Risk had positive impacts. Overall, the net impact is -4.7057, indicating a negative outcome for this customer.</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="BQ10" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1008" who made a purchase on September 2, 2024 through the Direct channel and belongs to the Consumer segment, the model score is 0.57. The top contributor to this score is Last Login, which had a positive impact of +1.45. This suggests that the customer's recent login activity was a significant factor in their decision to make a purchase. Overall, the net impact of all contributors was a positive +0.42, indicating that most factors contributed positively to the model score.</t>
+          <t>The model score for customer cust_1008 on 2024-09-02 is 0.5716, with a net impact of +0.4205. The dominant factor driving this positive outcome is the Last Login feature, which contributed +1.4516 to the overall score. This suggests that the customer's recent login activity had a significant and favorable influence on their behavior.</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="BQ11" t="inlineStr">
         <is>
-          <t>The top contributor to this customer's score is their NPS Score, which had a significant positive impact of +1.4215. This suggests that the customer has a very high level of satisfaction with our product or service. Additionally, the fact that they resulted in a purchase worth $852.84 and had a model score of 0.5958 indicates that they are a valuable customer. The overall net impact of their contributions is +0.7011, which suggests that their positive behaviors outweighed their negative ones.</t>
+          <t>The dominant factor driving the model score of 0.5958 is a positive NPS Score contribution of +1.4215, which accounts for approximately 5.6% of the overall impact. This suggests that customer satisfaction and loyalty have had a significant influence on the score. Additionally, Product Views (+1.4166) also contributed positively to the model score. The net impact is a positive +0.7011, indicating that the total positive contributions outweighed the negative ones.</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="BQ12" t="inlineStr">
         <is>
-          <t>The top contributor to the model score for this customer (cust_1010) is Usage Frequency, which had a positive impact of +1.4434. This suggests that the customer's frequent usage of our product or service was a key factor in their high model score. Additionally, other positive contributors included Revenue Potential and Device Type, indicating that the customer's potential to generate revenue and their device type also played a role in their score. Overall, the net impact of these contributions was +1.9124, indicating a strong positive influence on the model score.</t>
+          <t>The model score for this customer (cust_1010) is 0.7075, indicating a positive overall impact. The dominant feature driving this score is Usage Frequency, which contributed +1.4434 to the total score. This suggests that the customer's frequent usage of our product or service had a significant positive effect on their likelihood to make a purchase. Additionally, other positive contributors include Revenue Potential and Device Type, while Support Tickets was the top negative contributor with a -1.4290 impact. Overall, the net impact is +1.9124, indicating that the customer's behavior had a strong positive influence on their purchasing decision.</t>
         </is>
       </c>
     </row>
@@ -4119,8 +4119,7 @@
       </c>
       <c r="BQ13" t="inlineStr">
         <is>
-          <t>Here's a summary of the top factors that influenced this customer's score:
-The dominant factor in this case was the customer's Last Login, which had a significant negative impact (-1.4949). This suggests that the customer hasn't logged in recently, indicating a potential disengagement or lack of activity. Additionally, the positive contributions from Demo Requests (+1.3211) and Purchase History (+1.2767) were not enough to overcome this negative factor. Overall, the net impact was slightly positive (+0.2463), but the Last Login factor had a significant influence on the score.</t>
+          <t>The model score for this customer (cust_1011) is 0.5346, indicating a moderate likelihood of making a purchase. The dominant factor driving this score is the Last Login feature, which had a negative contribution value of -1.4949 and accounted for 7.7% of the overall dominance ratio. This suggests that the customer's lack of recent login activity has had a significant impact on their model score.</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4398,7 @@
       </c>
       <c r="BQ14" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1012" who interacted through Organic Search, the model score is 0.0599, indicating a relatively low influence on the overall score. The top contributors to this score are mostly negative, with API Calls being the dominant factor (-1.4834), making up about 7.2% of the total impact. This suggests that the customer's behavior in terms of API usage had a significant negative effect on their overall score.</t>
+          <t>The model score for this customer (cust_1012) is 0.0599, which is influenced by a net negative impact of -4.6548. The dominant factor contributing to this negative impact is API Calls, with a contribution value of -1.4834, accounting for approximately 7.2% of the total negative impact. This suggests that the customer's API usage patterns had a significant negative effect on their model score.</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4677,7 @@
       </c>
       <c r="BQ15" t="inlineStr">
         <is>
-          <t>The top contributor to the score for this customer, cust_1013, is Purchase History, which had a positive impact of +1.2524. This suggests that the customer's purchase history played a significant role in determining their score. In fact, the net impact of all contributors was +4.3916, indicating a strong overall positive influence. The dominant feature, Purchase History, accounted for 6.6% of the total contribution, further emphasizing its importance.</t>
+          <t>The model score for this customer (cust_1013) is 0.9538, indicating a strong positive outcome. The dominant factor driving this score is Purchase History (+1.2524), which accounts for approximately 6.6% of the overall net impact. This suggests that the customer's purchase history had a significant and positive influence on their behavior. Additionally, other factors such as Account Age (+1.2206) and Device Type (+1.1761) also contributed positively to the score, while Click Rate (-1.1359) and Session Duration (-1.1000) had negative impacts. Overall, the net impact is +4.3916, indicating a positive outcome.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4956,7 @@
       </c>
       <c r="BQ16" t="inlineStr">
         <is>
-          <t>The model score for this customer (cust_1014) is 0.3703, indicating a moderate influence on the overall score. The top contributor to this score is the Location Score, which had a negative impact of -1.4823. This suggests that the customer's location may have played a significant role in their behavior or preferences, resulting in a lower model score. Overall, the net impact of these contributions is a negative value of -1.5324, indicating that more factors had a negative influence than positive ones.</t>
+          <t>The model score for this customer (cust_1014) is 0.3703, which is influenced by a net negative impact of -1.5324. The dominant factor contributing to this score is the Location Score (-1.4823), accounting for approximately 7.1% of the total contribution. While there are some positive contributors, such as NPS Score (+1.3603) and Social Shares (+1.2145), the negative impact from Location Score and other factors like API Calls (-1.4129) and Last Login (-1.3073) outweighs the positives, resulting in a net negative score.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5235,7 @@
       </c>
       <c r="BQ17" t="inlineStr">
         <is>
-          <t>The top contributor to this customer's score is Email Opens, with a positive impact of +1.4422. This suggests that the customer's engagement with email campaigns had a significant influence on their overall score. In fact, the total positive contributions from email-related activities (+13.8828) far outweighed the negative contributions from other factors (-12.2770), resulting in a net impact of +1.6058. Overall, this customer's score was positively tilted, with a dominant factor like Email Opens playing a key role in their outcome.</t>
+          <t>The dominant factor driving the model score of 0.6874 was Email Opens, which contributed a positive value of +1.4422. This suggests that customers who engaged with emails were more likely to result in a purchase, as evidenced by the high resulted_in_purchase rate of 1.0000 and the resulting purchase value of $1261.60. The overall net impact of +1.6058 indicates a positive trend, with more positive contributors (+13.8828) than negative ones (-12.2770).</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5514,7 @@
       </c>
       <c r="BQ18" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1016" who made a purchase on May 16, 2025 through the Referral channel and belongs to the Enterprise segment, the model score is 0.99, indicating a high likelihood of conversion. The top contributor to this positive outcome was Session Duration, which had a significant impact of +1.39. This suggests that the customer's prolonged engagement with our platform played a crucial role in their decision to make a purchase. Overall, the net impact was positive, with a score of +5.29, indicating that the factors contributing to this outcome were more influential than those that detracted from it.</t>
+          <t>The model score for this customer (cust_1016) is 0.990, indicating a strong positive influence from various factors. The net impact of these contributors is a positive +5.2892, driven primarily by Session Duration (+1.3912), which accounts for approximately 6.5% of the overall dominance ratio. This suggests that the customer's session duration had a significant and positive impact on their purchase decision, resulting in a purchase value of $184.47.</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5793,7 @@
       </c>
       <c r="BQ19" t="inlineStr">
         <is>
-          <t>The top contributor to the model score for this customer is Lead Behavior, with a negative impact of 1.4620. This suggests that the customer's lead behavior had a significant influence on the overall score, pulling it down. In fact, the net impact of all contributors is slightly negative (-0.0502), indicating that the positive contributions from factors like Usage Frequency (+1.3039) and Product Views (+1.2589) were not enough to overcome the negative impact of Lead Behavior.</t>
+          <t>The model score for customer cust_1017 on 2025-06-01, driven by the Social channel and Enterprise segment, is 0.5101. The dominant factor contributing to this score is Lead Behavior (-1.4620), which had a significant negative impact. This was offset by positive contributions from Usage Frequency (+1.3039) and Product Views (+1.2589). Overall, the net impact of these factors was a small negative effect (-0.0502), indicating that while some aspects of this customer's behavior were beneficial, their lead behavior had a more significant detrimental influence.</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6072,7 @@
       </c>
       <c r="BQ20" t="inlineStr">
         <is>
-          <t>For the customer with ID "cust_1018" who interacted with our marketing campaign on July 23, 2025 through the Email channel and belongs to the Enterprise segment, the dominant factor that influenced their score was Plan Type, which had a positive contribution of +1.4899. This suggests that the type of plan they were considering had a significant impact on their overall score. While there were some negative contributors, such as Social Shares (-1.4483) and Email Opens (-0.9268), the positive influence of Plan Type outweighed these negatives, resulting in a net impact of -3.7971. Overall, this customer's score was driven by their consideration of different plan options, which had a significant bearing on their likelihood to make a purchase.</t>
+          <t>The model score for this customer (cust_1018) is 0.1451, which is influenced by a net negative impact of -3.7971. The dominant factor contributing to this score is Plan Type, with a positive value of +1.4899, accounting for 8.7% of the total contribution. This suggests that the customer's plan type had a significant positive impact on their model score.</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6351,7 @@
       </c>
       <c r="BQ21" t="inlineStr">
         <is>
-          <t>The score for this customer (cust_1019) was influenced by a mix of positive and negative factors, with the overall net impact being slightly negative (-4.3075). The dominant factor contributing to this score is Referral Source, which had a significant negative impact (-1.4632). This suggests that the customer's referral source may have played a role in their lower score. On the other hand, Lead Behavior and Plan Type both had positive contributions (+1.4415 and +1.3965 respectively), indicating that the customer's behavior and plan type were favorable factors. Overall, while there are some positive contributors, the negative impact of Referral Source was the most significant factor in determining this score.</t>
+          <t>The model score for this customer (cust_1019) is 0.0842, which is influenced by a net negative impact of -4.3075. The dominant factor contributing to this score is Referral Source (-1.4632), making up about 5.5% of the total contribution. This suggests that the customer's referral source had a significant negative impact on their model score.</t>
         </is>
       </c>
     </row>

</xml_diff>